<commit_message>
receipt machine origin api insertion
</commit_message>
<xml_diff>
--- a/app/backends/sveltekit/template/output.xlsx
+++ b/app/backends/sveltekit/template/output.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F6"/>
   <cols>
     <col min="2" max="2" customWidth="1" width="25"/>
     <col min="3" max="3" customWidth="1" width="30"/>
@@ -437,7 +437,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Sat Oct 18 2025 23:17:27 GMT+0100 (West Africa Standard Time)</v>
+        <v>Sun Oct 19 2025 17:50:25 GMT+0100 (West Africa Standard Time)</v>
       </c>
       <c r="C2" t="str">
         <v>Transportation</v>
@@ -446,7 +446,7 @@
         <v>20000</v>
       </c>
       <c r="E2" s="1">
-        <v>69150</v>
+        <v>5700</v>
       </c>
       <c r="F2" s="1" t="e">
         <f>D2 - E2</f>
@@ -457,16 +457,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Sat Oct 18 2025 23:17:27 GMT+0100 (West Africa Standard Time)</v>
+        <v>Sun Oct 19 2025 17:50:25 GMT+0100 (West Africa Standard Time)</v>
       </c>
       <c r="C3" t="str">
-        <v>Food and Provision</v>
+        <v xml:space="preserve">Food </v>
       </c>
       <c r="D3" s="1">
-        <v>100000</v>
+        <v>25000</v>
       </c>
       <c r="E3" s="1">
-        <v>13000</v>
+        <v>0</v>
       </c>
       <c r="F3" s="1" t="e">
         <f>D3 - E3</f>
@@ -477,32 +477,72 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Sat Oct 18 2025 23:17:27 GMT+0100 (West Africa Standard Time)</v>
+        <v>Sun Oct 19 2025 17:50:25 GMT+0100 (West Africa Standard Time)</v>
       </c>
       <c r="C4" t="str">
-        <v>Text Books</v>
+        <v>Network</v>
       </c>
       <c r="D4" s="1">
-        <v>80000</v>
+        <v>10000</v>
       </c>
       <c r="E4" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="F4" s="1" t="e">
         <f>D4 - E4</f>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Sun Oct 19 2025 17:50:25 GMT+0100 (West Africa Standard Time)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Electricity Bills</v>
+      </c>
+      <c r="D5" s="1">
+        <v>50000</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1" t="e">
+        <f>D5 - E5</f>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Sun Oct 19 2025 17:50:25 GMT+0100 (West Africa Standard Time)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Garbage Collector Bills</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3000</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1" t="e">
+        <f>D6 - E6</f>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I2"/>
   <cols>
     <col min="2" max="2" customWidth="1" width="25"/>
     <col min="3" max="3" customWidth="1" width="40"/>
@@ -548,299 +588,34 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Sat Oct 18 2025 23:43:15 GMT+0100 (West Africa Standard Time)</v>
+        <v>Wed Oct 22 2025 11:35:34 GMT+0100 (West Africa Standard Time)</v>
       </c>
       <c r="C2" t="str">
-        <v>Food and Provision</v>
+        <v>Transportation</v>
       </c>
       <c r="D2" t="str">
-        <v>First week Provision</v>
+        <v>Lorenting</v>
       </c>
       <c r="E2" s="1">
-        <v>3000</v>
+        <v>5700</v>
       </c>
       <c r="F2" s="1">
-        <v>97000</v>
+        <v>14300</v>
       </c>
       <c r="G2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Tue Oct 21 2025 12:22:38 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Transportation</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Eko Travels</v>
-      </c>
-      <c r="E3" s="1">
-        <v>20000</v>
-      </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Tue Oct 21 2025 12:23:54 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Transportation</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Abuja Travels</v>
-      </c>
-      <c r="E4" s="1">
-        <v>40000</v>
-      </c>
-      <c r="F4" s="1">
-        <v>-40000</v>
-      </c>
-      <c r="G4" s="1">
-        <v>40000</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Tue Oct 21 2025 12:25:56 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Transportation</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Enugu Travels</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1000</v>
-      </c>
-      <c r="F5" s="1">
-        <v>-41000</v>
-      </c>
-      <c r="G5" s="1">
-        <v>41000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Tue Oct 21 2025 12:27:06 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Transportation</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Ogun Travels</v>
-      </c>
-      <c r="E6" s="1">
-        <v>2000</v>
-      </c>
-      <c r="F6" s="1">
-        <v>-43000</v>
-      </c>
-      <c r="G6" s="1">
-        <v>43000</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Tue Oct 21 2025 12:45:50 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Transportation</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Break Fast Day One</v>
-      </c>
-      <c r="E7" s="1">
-        <v>6000</v>
-      </c>
-      <c r="F7" s="1">
-        <v>-49000</v>
-      </c>
-      <c r="G7" s="1">
-        <v>49000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Tue Oct 21 2025 12:47:43 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Transportation</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Dinner Day One</v>
-      </c>
-      <c r="E8" s="1">
-        <v>150</v>
-      </c>
-      <c r="F8" s="1">
-        <v>-49150</v>
-      </c>
-      <c r="G8" s="1">
-        <v>49150</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Tue Oct 21 2025 13:05:35 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Text Books</v>
-      </c>
-      <c r="D9" t="str">
-        <v>BanDoxi</v>
-      </c>
-      <c r="E9" s="1">
-        <v>100</v>
-      </c>
-      <c r="F9" s="1">
-        <v>79900</v>
-      </c>
-      <c r="G9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Tue Oct 21 2025 13:08:08 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Food and Provision</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Supper Day One</v>
-      </c>
-      <c r="E10" s="1">
-        <v>500</v>
-      </c>
-      <c r="F10" s="1">
-        <v>96500</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Tue Oct 21 2025 18:37:32 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Food and Provision</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Supper Day Two</v>
-      </c>
-      <c r="E11" s="1">
-        <v>500</v>
-      </c>
-      <c r="F11" s="1">
-        <v>96000</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0</v>
-      </c>
-      <c r="H11" t="str">
-        <v>Tue Oct 21 2025</v>
-      </c>
-      <c r="I11" t="str">
+      <c r="H2" t="str">
+        <v>Wed Oct 22 2025</v>
+      </c>
+      <c r="I2" t="str">
         <v>Manual Input</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Tue Oct 21 2025 18:41:15 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Food and Provision</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Dinner Day Two</v>
-      </c>
-      <c r="E12" s="1">
-        <v>6000</v>
-      </c>
-      <c r="F12" s="1">
-        <v>90000</v>
-      </c>
-      <c r="G12" s="1">
-        <v>0</v>
-      </c>
-      <c r="H12" t="str">
-        <v>24 may 2025</v>
-      </c>
-      <c r="I12" t="str">
-        <v>KUDA MICROFINANCE BANK</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Tue Oct 21 2025 18:56:17 GMT+0100 (West Africa Standard Time)</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Food and Provision</v>
-      </c>
-      <c r="D13" t="str">
-        <v>Lunch Day Three with Office</v>
-      </c>
-      <c r="E13" s="1">
-        <v>3000</v>
-      </c>
-      <c r="F13" s="1">
-        <v>87000</v>
-      </c>
-      <c r="G13" s="1">
-        <v>0</v>
-      </c>
-      <c r="H13" t="str">
-        <v>may 22, 2025</v>
-      </c>
-      <c r="I13" t="str">
-        <v>PALMPAY</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>